<commit_message>
Record the 12 October open on the live page.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/live_log/nifty_gap_log.xlsx
+++ b/live_log/nifty_gap_log.xlsx
@@ -568,14 +568,18 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Prediction locked</t>
+          <t>No call</t>
         </is>
       </c>
       <c r="G2" t="n">
         <v>22520.45</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>22593.2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.323</v>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>No call — not scored</t>
@@ -596,7 +600,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>No call. The S&amp;P move was 0.59%, under the 1% line.</t>
+          <t>No call. The S&amp;P move was 0.59%, under the 1% line. The open later moved 0.323% versus the previous close. This day is not counted.</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">

</xml_diff>

<commit_message>
Update the live gap log
</commit_message>
<xml_diff>
--- a/live_log/nifty_gap_log.xlsx
+++ b/live_log/nifty_gap_log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap test" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to read this" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gap test" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How to read this" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gap test'!$A$1:$Q$2</definedName>

</xml_diff>